<commit_message>
Update with Top-side cooling devices for GaN
</commit_message>
<xml_diff>
--- a/Switch Functions/GaN Data tf.xlsx
+++ b/Switch Functions/GaN Data tf.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MIT\Project\GE Vernova\Component\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1E7E01B-4CE4-45EB-A6BC-783DE761115B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{596F3C44-FF2D-44D2-A0DE-B43A0674A2BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="58">
   <si>
     <t>Part Number</t>
   </si>
@@ -159,6 +159,57 @@
   </si>
   <si>
     <t>Bottom</t>
+  </si>
+  <si>
+    <t>GNP2025TD-ZTR</t>
+  </si>
+  <si>
+    <t>Rohm GNP2025TD</t>
+  </si>
+  <si>
+    <t>GAN039-650NTBJ</t>
+  </si>
+  <si>
+    <t>Nexperia GAN039T</t>
+  </si>
+  <si>
+    <t>Top</t>
+  </si>
+  <si>
+    <t>TP65H030G4PRS-TR</t>
+  </si>
+  <si>
+    <t>Renesas 030G4PRS</t>
+  </si>
+  <si>
+    <t>IGLT65R035D2ATMA1</t>
+  </si>
+  <si>
+    <t>Infineon IGLT65R035</t>
+  </si>
+  <si>
+    <t>IGOT65R035D2AUMA1</t>
+  </si>
+  <si>
+    <t>Infineon IGOT65R035</t>
+  </si>
+  <si>
+    <t>IGT65R045D2ATMA1</t>
+  </si>
+  <si>
+    <t>Infineon IGT65R045</t>
+  </si>
+  <si>
+    <t>IGLT65R045D2ATMA1</t>
+  </si>
+  <si>
+    <t>Infineon IGLT65R045</t>
+  </si>
+  <si>
+    <t>IGOT65R045D2AUMA1</t>
+  </si>
+  <si>
+    <t>Infineon IGOT65R045</t>
   </si>
 </sst>
 </file>
@@ -195,7 +246,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -217,6 +268,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -273,7 +330,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -307,6 +364,12 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -589,7 +652,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X9"/>
+  <dimension ref="A1:X17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.26953125" customWidth="1"/>
@@ -722,7 +785,7 @@
         <v>6.3</v>
       </c>
       <c r="M2" s="7">
-        <f t="shared" ref="M2:M9" si="0">R2/X2</f>
+        <f t="shared" ref="M2:M17" si="0">R2/X2</f>
         <v>1.571428571428571</v>
       </c>
       <c r="N2" s="2">
@@ -738,7 +801,7 @@
         <v>1.9</v>
       </c>
       <c r="R2" s="2">
-        <f t="shared" ref="R2:R9" si="1">Q2-P2</f>
+        <f t="shared" ref="R2:R17" si="1">Q2-P2</f>
         <v>0.99999999999999989</v>
       </c>
       <c r="S2" s="2">
@@ -748,7 +811,7 @@
         <v>1.7</v>
       </c>
       <c r="U2" s="2">
-        <f t="shared" ref="U2:U9" si="2">V2+W2</f>
+        <f t="shared" ref="U2:U17" si="2">V2+W2</f>
         <v>3.3</v>
       </c>
       <c r="V2" s="2">
@@ -758,7 +821,7 @@
         <v>2</v>
       </c>
       <c r="X2" s="2">
-        <f t="shared" ref="X2:X9" si="3">(S2+T2)/(2*U2)</f>
+        <f t="shared" ref="X2:X17" si="3">(S2+T2)/(2*U2)</f>
         <v>0.63636363636363646</v>
       </c>
     </row>
@@ -1035,7 +1098,7 @@
       </c>
       <c r="M6" s="7">
         <f t="shared" si="0"/>
-        <v>1.7233333333333332</v>
+        <v>1.8267333333333329</v>
       </c>
       <c r="N6" s="2">
         <v>7.7</v>
@@ -1044,14 +1107,14 @@
         <v>3</v>
       </c>
       <c r="P6" s="2">
-        <v>0.7</v>
+        <v>0.66700000000000004</v>
       </c>
       <c r="Q6" s="2">
         <v>1.25</v>
       </c>
       <c r="R6" s="2">
         <f t="shared" si="1"/>
-        <v>0.55000000000000004</v>
+        <v>0.58299999999999996</v>
       </c>
       <c r="S6" s="2">
         <v>1.8</v>
@@ -1075,7 +1138,7 @@
       </c>
     </row>
     <row r="7" spans="1:24" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="13" t="s">
         <v>20</v>
       </c>
       <c r="B7" s="5" t="s">
@@ -1300,6 +1363,603 @@
       <c r="X9" s="2">
         <f t="shared" si="3"/>
         <v>0.15833333333333333</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="4">
+        <v>650</v>
+      </c>
+      <c r="D10" s="4">
+        <v>0.31</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G10" s="4">
+        <v>140</v>
+      </c>
+      <c r="H10" s="4">
+        <v>10.28</v>
+      </c>
+      <c r="I10" s="4">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="J10" s="2">
+        <v>5.8000000000000003E-2</v>
+      </c>
+      <c r="K10" s="2">
+        <v>150</v>
+      </c>
+      <c r="L10" s="7">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="M10" s="7">
+        <f t="shared" si="0"/>
+        <v>0.98181818181818203</v>
+      </c>
+      <c r="N10" s="2">
+        <v>13.2</v>
+      </c>
+      <c r="O10" s="2">
+        <v>6</v>
+      </c>
+      <c r="P10" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>0.9</v>
+      </c>
+      <c r="R10" s="2">
+        <f t="shared" si="1"/>
+        <v>0.15000000000000002</v>
+      </c>
+      <c r="S10" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="T10" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="U10" s="2">
+        <f t="shared" si="2"/>
+        <v>10.8</v>
+      </c>
+      <c r="V10" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="W10" s="2">
+        <v>10</v>
+      </c>
+      <c r="X10" s="2">
+        <f t="shared" si="3"/>
+        <v>0.15277777777777776</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+      <c r="A11" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="4">
+        <v>650</v>
+      </c>
+      <c r="D11" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G11" s="4">
+        <v>144</v>
+      </c>
+      <c r="H11" s="4">
+        <v>11.85</v>
+      </c>
+      <c r="I11" s="4">
+        <v>9.25</v>
+      </c>
+      <c r="J11" s="2">
+        <v>8.5999999999999993E-2</v>
+      </c>
+      <c r="K11" s="2">
+        <v>150</v>
+      </c>
+      <c r="L11" s="7">
+        <v>10</v>
+      </c>
+      <c r="M11" s="7">
+        <f t="shared" si="0"/>
+        <v>7.4468085106382951</v>
+      </c>
+      <c r="N11" s="2">
+        <v>26</v>
+      </c>
+      <c r="O11" s="2">
+        <v>10</v>
+      </c>
+      <c r="P11" s="2">
+        <v>7.4</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>10.199999999999999</v>
+      </c>
+      <c r="R11" s="2">
+        <f t="shared" si="1"/>
+        <v>2.7999999999999989</v>
+      </c>
+      <c r="S11" s="2">
+        <v>5.5</v>
+      </c>
+      <c r="T11" s="2">
+        <v>3.9</v>
+      </c>
+      <c r="U11" s="2">
+        <f t="shared" si="2"/>
+        <v>12.5</v>
+      </c>
+      <c r="V11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="W11" s="2">
+        <v>12</v>
+      </c>
+      <c r="X11" s="2">
+        <f t="shared" si="3"/>
+        <v>0.376</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="4">
+        <v>650</v>
+      </c>
+      <c r="D12" s="4">
+        <v>0.65</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G12" s="4">
+        <v>127</v>
+      </c>
+      <c r="H12" s="4">
+        <v>10</v>
+      </c>
+      <c r="I12" s="4">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="J12" s="2">
+        <v>6.2E-2</v>
+      </c>
+      <c r="K12" s="2">
+        <v>150</v>
+      </c>
+      <c r="L12" s="7">
+        <v>6.4</v>
+      </c>
+      <c r="M12" s="7">
+        <f t="shared" si="0"/>
+        <v>13.578947368421055</v>
+      </c>
+      <c r="N12" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="O12" s="2">
+        <v>12</v>
+      </c>
+      <c r="P12" s="2">
+        <v>6.25</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>8.4</v>
+      </c>
+      <c r="R12" s="2">
+        <f t="shared" si="1"/>
+        <v>2.1500000000000004</v>
+      </c>
+      <c r="S12" s="2">
+        <v>5.5</v>
+      </c>
+      <c r="T12" s="2">
+        <v>4</v>
+      </c>
+      <c r="U12" s="2">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
+      <c r="W12" s="2">
+        <v>30</v>
+      </c>
+      <c r="X12" s="2">
+        <f t="shared" si="3"/>
+        <v>0.15833333333333333</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" s="4">
+        <v>650</v>
+      </c>
+      <c r="D13" s="4">
+        <v>0.81</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G13" s="4">
+        <v>91</v>
+      </c>
+      <c r="H13" s="4">
+        <v>10</v>
+      </c>
+      <c r="I13" s="4">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="J13" s="2">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="K13" s="2">
+        <v>150</v>
+      </c>
+      <c r="L13" s="7">
+        <v>10</v>
+      </c>
+      <c r="M13" s="7">
+        <f t="shared" si="0"/>
+        <v>1.8267333333333329</v>
+      </c>
+      <c r="N13" s="2">
+        <v>7.7</v>
+      </c>
+      <c r="O13" s="2">
+        <v>3</v>
+      </c>
+      <c r="P13" s="2">
+        <v>0.66700000000000004</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>1.25</v>
+      </c>
+      <c r="R13" s="2">
+        <f t="shared" si="1"/>
+        <v>0.58299999999999996</v>
+      </c>
+      <c r="S13" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="T13" s="2">
+        <v>1.2</v>
+      </c>
+      <c r="U13" s="2">
+        <f t="shared" si="2"/>
+        <v>4.6999999999999993</v>
+      </c>
+      <c r="V13" s="2">
+        <v>1.4</v>
+      </c>
+      <c r="W13" s="2">
+        <v>3.3</v>
+      </c>
+      <c r="X13" s="2">
+        <f t="shared" si="3"/>
+        <v>0.31914893617021284</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="4">
+        <v>650</v>
+      </c>
+      <c r="D14" s="4">
+        <v>0.94</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G14" s="4">
+        <v>91</v>
+      </c>
+      <c r="H14" s="4">
+        <v>15.64</v>
+      </c>
+      <c r="I14" s="4">
+        <v>10.85</v>
+      </c>
+      <c r="J14" s="2">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="K14" s="2">
+        <v>150</v>
+      </c>
+      <c r="L14" s="7">
+        <v>10</v>
+      </c>
+      <c r="M14" s="7">
+        <f t="shared" si="0"/>
+        <v>1.8267333333333329</v>
+      </c>
+      <c r="N14" s="2">
+        <v>7.7</v>
+      </c>
+      <c r="O14" s="2">
+        <v>3</v>
+      </c>
+      <c r="P14" s="2">
+        <v>0.66700000000000004</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>1.25</v>
+      </c>
+      <c r="R14" s="2">
+        <f t="shared" si="1"/>
+        <v>0.58299999999999996</v>
+      </c>
+      <c r="S14" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="T14" s="2">
+        <v>1.2</v>
+      </c>
+      <c r="U14" s="2">
+        <f t="shared" si="2"/>
+        <v>4.6999999999999993</v>
+      </c>
+      <c r="V14" s="2">
+        <v>1.4</v>
+      </c>
+      <c r="W14" s="2">
+        <v>3.3</v>
+      </c>
+      <c r="X14" s="2">
+        <f t="shared" si="3"/>
+        <v>0.31914893617021284</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+      <c r="A15" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="4">
+        <v>650</v>
+      </c>
+      <c r="D15" s="4">
+        <v>0.95</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G15" s="4">
+        <v>72</v>
+      </c>
+      <c r="H15" s="4">
+        <v>10.275</v>
+      </c>
+      <c r="I15" s="4">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="J15" s="2">
+        <v>9.6000000000000002E-2</v>
+      </c>
+      <c r="K15" s="2">
+        <v>150</v>
+      </c>
+      <c r="L15" s="7">
+        <v>9</v>
+      </c>
+      <c r="M15" s="7">
+        <f t="shared" si="0"/>
+        <v>1.6189333333333333</v>
+      </c>
+      <c r="N15" s="2">
+        <v>6</v>
+      </c>
+      <c r="O15" s="2">
+        <v>3</v>
+      </c>
+      <c r="P15" s="2">
+        <v>0.53300000000000003</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>1</v>
+      </c>
+      <c r="R15" s="2">
+        <f t="shared" si="1"/>
+        <v>0.46699999999999997</v>
+      </c>
+      <c r="S15" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="T15" s="2">
+        <v>1.2</v>
+      </c>
+      <c r="U15" s="2">
+        <f t="shared" si="2"/>
+        <v>5.2</v>
+      </c>
+      <c r="V15" s="2">
+        <v>1.3</v>
+      </c>
+      <c r="W15" s="2">
+        <v>3.9</v>
+      </c>
+      <c r="X15" s="2">
+        <f t="shared" si="3"/>
+        <v>0.28846153846153844</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+      <c r="A16" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="4">
+        <v>650</v>
+      </c>
+      <c r="D16" s="4">
+        <v>1</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G16" s="4">
+        <v>72</v>
+      </c>
+      <c r="H16" s="4">
+        <v>10</v>
+      </c>
+      <c r="I16" s="4">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="J16" s="2">
+        <v>9.6000000000000002E-2</v>
+      </c>
+      <c r="K16" s="2">
+        <v>150</v>
+      </c>
+      <c r="L16" s="7">
+        <v>9</v>
+      </c>
+      <c r="M16" s="7">
+        <f t="shared" si="0"/>
+        <v>1.6189333333333333</v>
+      </c>
+      <c r="N16" s="2">
+        <v>6</v>
+      </c>
+      <c r="O16" s="2">
+        <v>3</v>
+      </c>
+      <c r="P16" s="2">
+        <v>0.53300000000000003</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>1</v>
+      </c>
+      <c r="R16" s="2">
+        <f t="shared" si="1"/>
+        <v>0.46699999999999997</v>
+      </c>
+      <c r="S16" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="T16" s="2">
+        <v>1.2</v>
+      </c>
+      <c r="U16" s="2">
+        <f t="shared" si="2"/>
+        <v>5.2</v>
+      </c>
+      <c r="V16" s="2">
+        <v>1.3</v>
+      </c>
+      <c r="W16" s="2">
+        <v>3.9</v>
+      </c>
+      <c r="X16" s="2">
+        <f t="shared" si="3"/>
+        <v>0.28846153846153844</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" s="4">
+        <v>650</v>
+      </c>
+      <c r="D17" s="4">
+        <v>1.2</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G17" s="4">
+        <v>72</v>
+      </c>
+      <c r="H17" s="4">
+        <v>15.64</v>
+      </c>
+      <c r="I17" s="4">
+        <v>10.85</v>
+      </c>
+      <c r="J17" s="2">
+        <v>9.6000000000000002E-2</v>
+      </c>
+      <c r="K17" s="2">
+        <v>150</v>
+      </c>
+      <c r="L17" s="7">
+        <v>9</v>
+      </c>
+      <c r="M17" s="7">
+        <f t="shared" si="0"/>
+        <v>1.6189333333333333</v>
+      </c>
+      <c r="N17" s="2">
+        <v>6</v>
+      </c>
+      <c r="O17" s="2">
+        <v>3</v>
+      </c>
+      <c r="P17" s="2">
+        <v>0.53300000000000003</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>1</v>
+      </c>
+      <c r="R17" s="2">
+        <f t="shared" si="1"/>
+        <v>0.46699999999999997</v>
+      </c>
+      <c r="S17" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="T17" s="2">
+        <v>1.2</v>
+      </c>
+      <c r="U17" s="2">
+        <f t="shared" si="2"/>
+        <v>5.2</v>
+      </c>
+      <c r="V17" s="2">
+        <v>1.3</v>
+      </c>
+      <c r="W17" s="2">
+        <v>3.9</v>
+      </c>
+      <c r="X17" s="2">
+        <f t="shared" si="3"/>
+        <v>0.28846153846153844</v>
       </c>
     </row>
   </sheetData>
@@ -1315,6 +1975,14 @@
     <hyperlink ref="B9" r:id="rId6" xr:uid="{9BF96118-FA77-4AA4-99CC-6FEB15379AFF}"/>
     <hyperlink ref="B2" r:id="rId7" xr:uid="{195B1C28-C3DF-4D3A-919D-115D1FB12604}"/>
     <hyperlink ref="B4" r:id="rId8" xr:uid="{A3A31E43-474D-4BD8-8613-CDDAF7E623D3}"/>
+    <hyperlink ref="B10" r:id="rId9" xr:uid="{3661E7B8-221B-432A-AD1D-C831D0C4CBA1}"/>
+    <hyperlink ref="B11" r:id="rId10" xr:uid="{9FE97FA5-89A7-456E-8502-AE5A6DCCBAAC}"/>
+    <hyperlink ref="B12" r:id="rId11" xr:uid="{415BFA58-79DB-4EA6-8430-5CEB9B5AF7D6}"/>
+    <hyperlink ref="B13" r:id="rId12" xr:uid="{B485EA92-93D0-4B32-844A-296EC4364521}"/>
+    <hyperlink ref="B14" r:id="rId13" xr:uid="{D8D21754-68AE-4A96-85D5-E765578A6996}"/>
+    <hyperlink ref="B15" r:id="rId14" xr:uid="{9418C3E7-1642-452E-9870-3956435196C4}"/>
+    <hyperlink ref="B16" r:id="rId15" xr:uid="{7D3CE121-093D-4193-8971-070CB236ED6D}"/>
+    <hyperlink ref="B17" r:id="rId16" xr:uid="{CCBB248E-20BD-4A2E-8604-93ED89D2CAC6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update with new thermal interface
</commit_message>
<xml_diff>
--- a/Switch Functions/GaN Data tf.xlsx
+++ b/Switch Functions/GaN Data tf.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MIT\Project\GE Vernova\Github\Switch Functions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6366CBC2-8970-48B7-A068-5A4654DE4A4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B92A4034-08F7-4FD4-B1AC-AEE08ED1198C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="61">
   <si>
     <t>Part Number</t>
   </si>
@@ -216,13 +216,16 @@
   </si>
   <si>
     <t>IGOT65R025D2AUMA1</t>
+  </si>
+  <si>
+    <t>Pin_Area</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -248,6 +251,17 @@
       <u/>
       <sz val="11"/>
       <color rgb="FF0563C1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -336,7 +350,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -376,6 +390,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -658,7 +678,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X18"/>
+  <dimension ref="A1:Y18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.26953125" customWidth="1"/>
@@ -676,10 +696,10 @@
     <col min="15" max="15" width="8.7265625" style="2"/>
     <col min="17" max="18" width="8.7265625" style="2"/>
     <col min="20" max="20" width="8.7265625" style="2"/>
-    <col min="22" max="24" width="8.7265625" style="2"/>
+    <col min="22" max="25" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>19</v>
       </c>
@@ -752,8 +772,11 @@
       <c r="X1" s="10" t="s">
         <v>38</v>
       </c>
+      <c r="Y1" s="10" t="s">
+        <v>60</v>
+      </c>
     </row>
-    <row r="2" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>26</v>
       </c>
@@ -830,8 +853,12 @@
         <f t="shared" ref="X2:X18" si="3">(S2+T2)/(2*U2)</f>
         <v>0.63636363636363646</v>
       </c>
+      <c r="Y2" s="2">
+        <f>(0.7+0.6)*9.9</f>
+        <v>12.87</v>
+      </c>
     </row>
-    <row r="3" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
         <v>25</v>
       </c>
@@ -908,8 +935,11 @@
         <f t="shared" si="3"/>
         <v>0.44339622641509435</v>
       </c>
+      <c r="Y3" s="2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>27</v>
       </c>
@@ -986,8 +1016,11 @@
         <f t="shared" si="3"/>
         <v>0.63636363636363646</v>
       </c>
+      <c r="Y4" s="2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
         <v>22</v>
       </c>
@@ -1032,7 +1065,7 @@
         <v>11</v>
       </c>
       <c r="O5" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P5" s="2">
         <v>1</v>
@@ -1064,8 +1097,12 @@
         <f t="shared" si="3"/>
         <v>0.51724137931034475</v>
       </c>
+      <c r="Y5" s="2">
+        <f>(11.475-10.275)*9.7</f>
+        <v>11.639999999999992</v>
+      </c>
     </row>
-    <row r="6" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
         <v>21</v>
       </c>
@@ -1110,7 +1147,7 @@
         <v>7.7</v>
       </c>
       <c r="O6" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P6" s="2">
         <v>0.66700000000000004</v>
@@ -1142,8 +1179,12 @@
         <f t="shared" si="3"/>
         <v>0.31914893617021284</v>
       </c>
+      <c r="Y6" s="2">
+        <f>(11.475-10.275)*9.7</f>
+        <v>11.639999999999992</v>
+      </c>
     </row>
-    <row r="7" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
         <v>20</v>
       </c>
@@ -1220,8 +1261,12 @@
         <f t="shared" si="3"/>
         <v>0.376</v>
       </c>
+      <c r="Y7" s="2">
+        <f>(11.85-9.25)*11.85</f>
+        <v>30.809999999999995</v>
+      </c>
     </row>
-    <row r="8" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
         <v>24</v>
       </c>
@@ -1231,7 +1276,7 @@
       <c r="C8" s="4">
         <v>650</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="14">
         <v>0.65</v>
       </c>
       <c r="E8" s="4" t="s">
@@ -1295,8 +1340,12 @@
         <f t="shared" si="3"/>
         <v>0.15833333333333333</v>
       </c>
+      <c r="Y8" s="2">
+        <f>(11.48-10.28)*9.7</f>
+        <v>11.640000000000009</v>
+      </c>
     </row>
-    <row r="9" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
         <v>23</v>
       </c>
@@ -1306,7 +1355,7 @@
       <c r="C9" s="4">
         <v>650</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="14">
         <v>0.8</v>
       </c>
       <c r="E9" s="4" t="s">
@@ -1370,8 +1419,12 @@
         <f t="shared" si="3"/>
         <v>0.15833333333333333</v>
       </c>
+      <c r="Y9" s="2">
+        <f>(11.48-10.28)*9.7</f>
+        <v>11.640000000000009</v>
+      </c>
     </row>
-    <row r="10" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>42</v>
       </c>
@@ -1381,8 +1434,8 @@
       <c r="C10" s="4">
         <v>650</v>
       </c>
-      <c r="D10" s="4">
-        <v>0.31</v>
+      <c r="D10" s="15">
+        <v>0.43</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>40</v>
@@ -1445,8 +1498,12 @@
         <f t="shared" si="3"/>
         <v>0.15277777777777776</v>
       </c>
+      <c r="Y10" s="2">
+        <f>(11.48-10.28)*9.7</f>
+        <v>11.640000000000009</v>
+      </c>
     </row>
-    <row r="11" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
         <v>44</v>
       </c>
@@ -1520,8 +1577,12 @@
         <f t="shared" si="3"/>
         <v>0.376</v>
       </c>
+      <c r="Y11" s="2">
+        <f>(11.85-9.25)*11.85</f>
+        <v>30.809999999999995</v>
+      </c>
     </row>
-    <row r="12" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
         <v>47</v>
       </c>
@@ -1531,7 +1592,7 @@
       <c r="C12" s="4">
         <v>650</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="14">
         <v>0.65</v>
       </c>
       <c r="E12" s="4" t="s">
@@ -1592,8 +1653,12 @@
         <f t="shared" si="3"/>
         <v>0.15833333333333333</v>
       </c>
+      <c r="Y12" s="2">
+        <f>(14.8-10)*9.7</f>
+        <v>46.56</v>
+      </c>
     </row>
-    <row r="13" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
         <v>49</v>
       </c>
@@ -1635,7 +1700,7 @@
         <v>7.7</v>
       </c>
       <c r="O13" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P13" s="2">
         <v>0.66700000000000004</v>
@@ -1667,8 +1732,12 @@
         <f t="shared" si="3"/>
         <v>0.31914893617021284</v>
       </c>
+      <c r="Y13" s="2">
+        <f>(14.8-10)*9.7</f>
+        <v>46.56</v>
+      </c>
     </row>
-    <row r="14" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
         <v>51</v>
       </c>
@@ -1710,7 +1779,7 @@
         <v>7.7</v>
       </c>
       <c r="O14" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P14" s="2">
         <v>0.66700000000000004</v>
@@ -1742,8 +1811,12 @@
         <f t="shared" si="3"/>
         <v>0.31914893617021284</v>
       </c>
+      <c r="Y14" s="2">
+        <f>(13.9-10.85)*15.64</f>
+        <v>47.702000000000012</v>
+      </c>
     </row>
-    <row r="15" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
         <v>53</v>
       </c>
@@ -1785,7 +1858,7 @@
         <v>6</v>
       </c>
       <c r="O15" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P15" s="2">
         <v>0.53300000000000003</v>
@@ -1817,8 +1890,12 @@
         <f t="shared" si="3"/>
         <v>0.28846153846153844</v>
       </c>
+      <c r="Y15" s="2">
+        <f>(11.475-10.275)*9.7</f>
+        <v>11.639999999999992</v>
+      </c>
     </row>
-    <row r="16" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="8" t="s">
         <v>55</v>
       </c>
@@ -1860,7 +1937,7 @@
         <v>6</v>
       </c>
       <c r="O16" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P16" s="2">
         <v>0.53300000000000003</v>
@@ -1892,8 +1969,12 @@
         <f t="shared" si="3"/>
         <v>0.28846153846153844</v>
       </c>
+      <c r="Y16" s="2">
+        <f>(14.8-10)*9.7</f>
+        <v>46.56</v>
+      </c>
     </row>
-    <row r="17" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="8" t="s">
         <v>57</v>
       </c>
@@ -1935,7 +2016,7 @@
         <v>6</v>
       </c>
       <c r="O17" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P17" s="2">
         <v>0.53300000000000003</v>
@@ -1967,8 +2048,12 @@
         <f t="shared" si="3"/>
         <v>0.28846153846153844</v>
       </c>
+      <c r="Y17" s="2">
+        <f>(13.9-10.85)*15.64</f>
+        <v>47.702000000000012</v>
+      </c>
     </row>
-    <row r="18" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="8" t="s">
         <v>58</v>
       </c>
@@ -2010,7 +2095,7 @@
         <v>11</v>
       </c>
       <c r="O18" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P18" s="2">
         <v>1</v>
@@ -2041,6 +2126,10 @@
       <c r="X18" s="2">
         <f t="shared" si="3"/>
         <v>0.51724137931034475</v>
+      </c>
+      <c r="Y18" s="2">
+        <f>(13.9-10.85)*15.64</f>
+        <v>47.702000000000012</v>
       </c>
     </row>
   </sheetData>
@@ -2067,5 +2156,6 @@
     <hyperlink ref="B18" r:id="rId17" xr:uid="{F9225203-FC35-489F-996F-35C0871FC8D7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId18"/>
 </worksheet>
 </file>
</xml_diff>